<commit_message>
V8.1: temporizador/cronómetro, Full Body A/B de complemento y revisión visual
- Registrar: apartado de temporizador (1:00-4:00, ±15 s) y cronómetro;
  persiste al cambiar de sección o recargar; vibra y suena al terminar.
- Complemento - Full Body A/B por semana: cubren exactamente las series
  que faltan para el objetivo semanal (prioridad isquios). No cambian la
  rutina, series, reps, RIR ni objetivos existentes; se agregan también
  a datos ya guardados sin pisar ediciones.
- Plantilla Excel con los nuevos días.
- Botón primario con más contraste (auditoría visual en 3 tamaños).
- Pruebas: rutina original intacta, full body sin pasarse del objetivo,
  migración y temporizador (15/15).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuTVv6A6wSwyNRAbEh4sKC
</commit_message>
<xml_diff>
--- a/Plantilla_Prime_OS_V7.xlsx
+++ b/Plantilla_Prime_OS_V7.xlsx
@@ -2731,7 +2731,7 @@
       <formula1>Listas!$C$2:$C$8</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Listas!$E$2:$E$8</formula1>
+      <formula1>Listas!$E$2:$E$10</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Listas!$A$2:$A$16</formula1>
@@ -8238,7 +8238,7 @@
       <formula1>Listas!$C$2:$C$8</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Listas!$E$2:$E$8</formula1>
+      <formula1>Listas!$E$2:$E$10</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Listas!$A$2:$A$16</formula1>
@@ -8945,6 +8945,11 @@
           <t>bíceps</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Complemento - Full Body A</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8952,6 +8957,11 @@
           <t>tríceps</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Complemento - Full Body B</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V8.2: día y sesión separados, reloj flotante y actualizaciones sin mezclas
- Selector de día (Lunes-Domingo) y selector de sesión (Lower A/B,
  Upper A/B, Full Body A/B, Cardio, Trote, Descanso). Full Body sale de la
  lista de días. Las sesiones y ejercicios semana a semana no cambian.
- Temporizador/cronómetro como botón flotante "Reloj" con panel compacto
  y botón para cerrar; muestra el tiempo mientras corre.
- Ejercicio agregado aparece al inicio (Registrar y Rutina Base).
- Franja Sistema/Objetivo/Debilidad al final de la página.
- Service worker: caché exacta por versión, activación inmediata y
  recarga única desde index.html; antes una versión nueva podía cargar
  CSS y plan de la anterior.
- Pruebas 17/17 y auditoría visual sin problemas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuTVv6A6wSwyNRAbEh4sKC
</commit_message>
<xml_diff>
--- a/Plantilla_Prime_OS_V7.xlsx
+++ b/Plantilla_Prime_OS_V7.xlsx
@@ -8947,7 +8947,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Complemento - Full Body A</t>
+          <t>Full Body A</t>
         </is>
       </c>
     </row>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Complemento - Full Body B</t>
+          <t>Full Body B</t>
         </is>
       </c>
     </row>

</xml_diff>